<commit_message>
EngineData와 FacilityData에 Icon 이름 컬럼 추가
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Engine_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Engine_Data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="68">
   <si>
     <t>ID</t>
   </si>
@@ -231,6 +231,30 @@
   </si>
   <si>
     <t>0,0;0,1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Icon</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_test</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_test</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_test</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_test</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_test</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -974,14 +998,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="표1" displayName="표1" ref="A1:H23" totalsRowShown="0">
-  <autoFilter ref="A1:H23"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="표1" displayName="표1" ref="A1:I23" totalsRowShown="0">
+  <autoFilter ref="A1:I23"/>
+  <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="8" name="Name"/>
     <tableColumn id="6" name="EngineId"/>
     <tableColumn id="5" name="DisplayName"/>
     <tableColumn id="2" name="Type"/>
+    <tableColumn id="9" name="Icon"/>
     <tableColumn id="3" name="Level"/>
     <tableColumn id="4" name="Coordinates"/>
     <tableColumn id="7" name="Desc"/>
@@ -1253,17 +1278,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.75" customWidth="1"/>
     <col min="3" max="3" width="18.375" customWidth="1"/>
     <col min="4" max="4" width="13.375" customWidth="1"/>
-    <col min="7" max="7" width="35.875" customWidth="1"/>
+    <col min="6" max="6" width="18.375" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
     <col min="8" max="8" width="34.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1280,16 +1306,19 @@
         <v>1</v>
       </c>
       <c r="F1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>201001</v>
       </c>
@@ -1305,17 +1334,20 @@
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2">
         <v>1</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>55</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>201002</v>
       </c>
@@ -1331,17 +1363,20 @@
       <c r="E3" t="s">
         <v>4</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3">
         <v>2</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>56</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>201003</v>
       </c>
@@ -1357,17 +1392,20 @@
       <c r="E4" t="s">
         <v>4</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>58</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>201004</v>
       </c>
@@ -1383,17 +1421,20 @@
       <c r="E5" t="s">
         <v>4</v>
       </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="F5" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5" t="s">
         <v>60</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>202001</v>
       </c>
@@ -1409,17 +1450,20 @@
       <c r="E6" t="s">
         <v>4</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6">
         <v>1</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>55</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>202002</v>
       </c>
@@ -1435,17 +1479,20 @@
       <c r="E7" t="s">
         <v>4</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G7">
         <v>2</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>61</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>202003</v>
       </c>
@@ -1461,17 +1508,20 @@
       <c r="E8" t="s">
         <v>4</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8">
         <v>3</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>57</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>202004</v>
       </c>
@@ -1487,17 +1537,20 @@
       <c r="E9" t="s">
         <v>4</v>
       </c>
-      <c r="F9">
-        <v>4</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="F9" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9">
+        <v>4</v>
+      </c>
+      <c r="H9" t="s">
         <v>59</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>203001</v>
       </c>
@@ -1513,17 +1566,20 @@
       <c r="E10" t="s">
         <v>4</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10">
         <v>1</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>55</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>203002</v>
       </c>
@@ -1539,17 +1595,20 @@
       <c r="E11" t="s">
         <v>4</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11">
         <v>2</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>56</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>203003</v>
       </c>
@@ -1565,17 +1624,20 @@
       <c r="E12" t="s">
         <v>4</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12">
         <v>3</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>58</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>203004</v>
       </c>
@@ -1591,17 +1653,20 @@
       <c r="E13" t="s">
         <v>4</v>
       </c>
-      <c r="F13">
-        <v>4</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="F13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13">
+        <v>4</v>
+      </c>
+      <c r="H13" t="s">
         <v>60</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>204001</v>
       </c>
@@ -1617,17 +1682,20 @@
       <c r="E14" t="s">
         <v>4</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14">
         <v>1</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>55</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>204002</v>
       </c>
@@ -1643,17 +1711,20 @@
       <c r="E15" t="s">
         <v>4</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15">
         <v>2</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>56</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>204003</v>
       </c>
@@ -1669,17 +1740,20 @@
       <c r="E16" t="s">
         <v>4</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G16">
         <v>3</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>58</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>204004</v>
       </c>
@@ -1695,17 +1769,20 @@
       <c r="E17" t="s">
         <v>4</v>
       </c>
-      <c r="F17">
-        <v>4</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="F17" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17" t="s">
         <v>60</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>205001</v>
       </c>
@@ -1721,17 +1798,20 @@
       <c r="E18" t="s">
         <v>4</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G18">
         <v>1</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>55</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>205002</v>
       </c>
@@ -1747,17 +1827,20 @@
       <c r="E19" t="s">
         <v>4</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G19">
         <v>2</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>56</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>205003</v>
       </c>
@@ -1773,17 +1856,20 @@
       <c r="E20" t="s">
         <v>4</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20">
         <v>3</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>58</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>205004</v>
       </c>
@@ -1799,17 +1885,20 @@
       <c r="E21" t="s">
         <v>4</v>
       </c>
-      <c r="F21">
-        <v>4</v>
-      </c>
-      <c r="G21" t="s">
+      <c r="F21" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
+      <c r="H21" t="s">
         <v>60</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>211001</v>
       </c>
@@ -1821,15 +1910,18 @@
       <c r="E22" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G22" s="2">
         <v>1</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="H22" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I22" s="7"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>211002</v>
       </c>
@@ -1841,13 +1933,16 @@
       <c r="E23" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" s="6">
         <v>2</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="H23" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>

</xml_diff>

<commit_message>
엔진 formation / sprite / color 변경
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Engine_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Engine_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koseonghyeon\Desktop\Drill_Game\Drill_game\Assets\100_Data\XlsxFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0951BAD-7CB4-49C9-A441-FEE2D9816647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19FF288-156D-4012-8028-E01CC1F46721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="118">
   <si>
     <t>Type</t>
   </si>
@@ -387,6 +387,52 @@
   </si>
   <si>
     <t>보라 엔진 Lv.7</t>
+  </si>
+  <si>
+    <t>YellowEngine_5</t>
+  </si>
+  <si>
+    <t>노랑 엔진 Lv.5</t>
+  </si>
+  <si>
+    <t>YellowEngine_6</t>
+  </si>
+  <si>
+    <t>노랑 엔진 Lv.6</t>
+  </si>
+  <si>
+    <t>YellowEngine_7</t>
+  </si>
+  <si>
+    <t>노랑 엔진 Lv.7</t>
+  </si>
+  <si>
+    <t>0,0;0,1;1,0</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>2,2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0;0,1;1,0;1,1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0;0,1;1,0;1,1;0,2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0;0,1;1,0;1,1;0,2;1,2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0;0,1;1,0;1,1;0,2;1,2;0,3</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>2,4</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1100,8 +1146,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표1" displayName="표1" ref="A1:M34" totalsRowShown="0">
-  <autoFilter ref="A1:M34" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표1" displayName="표1" ref="A1:M37" totalsRowShown="0">
+  <autoFilter ref="A1:M37" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Name"/>
@@ -1384,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.75" customWidth="1"/>
@@ -1544,7 +1590,7 @@
         <v>3</v>
       </c>
       <c r="H4" t="s">
-        <v>51</v>
+        <v>111</v>
       </c>
       <c r="I4" t="s">
         <v>26</v>
@@ -1556,10 +1602,10 @@
         <v>1000</v>
       </c>
       <c r="L4" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="M4" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -1585,7 +1631,7 @@
         <v>4</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="I5" t="s">
         <v>26</v>
@@ -1597,10 +1643,10 @@
         <v>1000</v>
       </c>
       <c r="L5" t="s">
-        <v>70</v>
+        <v>112</v>
       </c>
       <c r="M5" t="s">
-        <v>73</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -1625,8 +1671,17 @@
       <c r="G6">
         <v>5</v>
       </c>
+      <c r="H6" t="s">
+        <v>114</v>
+      </c>
       <c r="I6" t="s">
         <v>26</v>
+      </c>
+      <c r="L6" t="s">
+        <v>70</v>
+      </c>
+      <c r="M6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -1651,8 +1706,17 @@
       <c r="G7">
         <v>6</v>
       </c>
+      <c r="H7" t="s">
+        <v>115</v>
+      </c>
       <c r="I7" t="s">
         <v>26</v>
+      </c>
+      <c r="L7" t="s">
+        <v>70</v>
+      </c>
+      <c r="M7" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -1677,8 +1741,17 @@
       <c r="G8">
         <v>7</v>
       </c>
+      <c r="H8" t="s">
+        <v>116</v>
+      </c>
       <c r="I8" t="s">
         <v>26</v>
+      </c>
+      <c r="L8" t="s">
+        <v>117</v>
+      </c>
+      <c r="M8" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -2572,39 +2645,117 @@
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A34" s="1">
+      <c r="A34">
+        <v>205005</v>
+      </c>
+      <c r="B34" t="s">
+        <v>105</v>
+      </c>
+      <c r="C34">
+        <v>205</v>
+      </c>
+      <c r="D34" t="s">
+        <v>106</v>
+      </c>
+      <c r="E34" t="s">
+        <v>78</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G34">
+        <v>5</v>
+      </c>
+      <c r="I34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>205006</v>
+      </c>
+      <c r="B35" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35">
+        <v>205</v>
+      </c>
+      <c r="D35" t="s">
+        <v>108</v>
+      </c>
+      <c r="E35" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G35">
+        <v>6</v>
+      </c>
+      <c r="I35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>205007</v>
+      </c>
+      <c r="B36" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36">
+        <v>205</v>
+      </c>
+      <c r="D36" t="s">
+        <v>110</v>
+      </c>
+      <c r="E36" t="s">
+        <v>78</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G36">
+        <v>7</v>
+      </c>
+      <c r="I36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
         <v>210001</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B37" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C34" s="2">
+      <c r="C37" s="2">
         <v>2001</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G34" s="2">
+      <c r="G37" s="2">
         <v>1</v>
       </c>
-      <c r="H34" t="s">
+      <c r="H37" t="s">
         <v>48</v>
       </c>
-      <c r="I34" s="5" t="s">
+      <c r="I37" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
-      <c r="L34" t="s">
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" t="s">
         <v>67</v>
       </c>
-      <c r="M34" t="s">
+      <c r="M37" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>